<commit_message>
feat: support nullable prices for hidden products and update cleaning product pricing and barcodes from PDF
</commit_message>
<xml_diff>
--- a/product-data/master/enJoyful_Master_Catalog.xlsx
+++ b/product-data/master/enJoyful_Master_Catalog.xlsx
@@ -526,7 +526,7 @@
         <v>200ml, 500ml</v>
       </c>
       <c r="H2" t="str">
-        <v>200ml:—  500ml:—</v>
+        <v>200ml:23.29  500ml:31.39</v>
       </c>
       <c r="I2" t="str">
         <v>baby-lotion</v>
@@ -561,7 +561,7 @@
         <v>50ml, 100ml</v>
       </c>
       <c r="H3" t="str">
-        <v>50ml:—  100ml:—</v>
+        <v>50ml:16.88  100ml:20.59</v>
       </c>
       <c r="I3" t="str">
         <v>baby-rash-cream</v>
@@ -596,7 +596,7 @@
         <v>75gm</v>
       </c>
       <c r="H4" t="str">
-        <v>75gm:—</v>
+        <v>75gm:11.48</v>
       </c>
       <c r="I4" t="str">
         <v>baby-soap</v>
@@ -631,7 +631,7 @@
         <v>200gm, 400gm</v>
       </c>
       <c r="H5" t="str">
-        <v>200gm:—  400gm:—</v>
+        <v>200gm:18.23  400gm:32.4</v>
       </c>
       <c r="I5" t="str">
         <v>baby-talc</v>
@@ -666,7 +666,7 @@
         <v>300ml, 500ml</v>
       </c>
       <c r="H6" t="str">
-        <v>300ml:—  500ml:—</v>
+        <v>300ml:25.65  500ml:31.39</v>
       </c>
       <c r="I6" t="str">
         <v>baby-wash</v>
@@ -701,7 +701,7 @@
         <v>100ml, 350ml</v>
       </c>
       <c r="H7" t="str">
-        <v>100ml:—  350ml:—</v>
+        <v>100ml:9.79  350ml:21.6</v>
       </c>
       <c r="I7" t="str">
         <v>almond-body-lotion</v>
@@ -736,7 +736,7 @@
         <v>100ml</v>
       </c>
       <c r="H8" t="str">
-        <v>100ml:—</v>
+        <v>100ml:9.79</v>
       </c>
       <c r="I8" t="str">
         <v>almond-moisturising-cream</v>
@@ -771,7 +771,7 @@
         <v>500ml</v>
       </c>
       <c r="H9" t="str">
-        <v>500ml:—</v>
+        <v>500ml:24.3</v>
       </c>
       <c r="I9" t="str">
         <v>aloe-bliss-shower-gel</v>
@@ -806,7 +806,7 @@
         <v>100ml, 400ml</v>
       </c>
       <c r="H10" t="str">
-        <v>100ml:—  400ml:—</v>
+        <v>100ml:8.78  400ml:19.24</v>
       </c>
       <c r="I10" t="str">
         <v>aloe-calm-shampoo</v>
@@ -841,7 +841,7 @@
         <v>100ml, 350ml</v>
       </c>
       <c r="H11" t="str">
-        <v>100ml:—  350ml:—</v>
+        <v>100ml:8.78  350ml:22.28</v>
       </c>
       <c r="I11" t="str">
         <v>aloevera-body-lotion</v>
@@ -876,7 +876,7 @@
         <v>25gm, 60gm</v>
       </c>
       <c r="H12" t="str">
-        <v>25gm:—  60gm:—</v>
+        <v>25gm:12.49  60gm:17.89</v>
       </c>
       <c r="I12" t="str">
         <v>aloevera-hair-removal-cream</v>
@@ -911,7 +911,7 @@
         <v>100ml, 400ml</v>
       </c>
       <c r="H13" t="str">
-        <v>100ml:—  400ml:—</v>
+        <v>100ml:8.78  400ml:18.23</v>
       </c>
       <c r="I13" t="str">
         <v>bamboo-balance-shampoo</v>
@@ -946,7 +946,7 @@
         <v>100ml, 400ml</v>
       </c>
       <c r="H14" t="str">
-        <v>100ml:—  400ml:—</v>
+        <v>100ml:8.78  400ml:21.6</v>
       </c>
       <c r="I14" t="str">
         <v>botanical-deep-clean-shampoo</v>
@@ -981,7 +981,7 @@
         <v>500ml</v>
       </c>
       <c r="H15" t="str">
-        <v>500ml:—</v>
+        <v>500ml:24.3</v>
       </c>
       <c r="I15" t="str">
         <v>c-glow-shower-gel</v>
@@ -1013,10 +1013,10 @@
         <v>1</v>
       </c>
       <c r="G16" t="str">
-        <v>100gm</v>
+        <v>100ml</v>
       </c>
       <c r="H16" t="str">
-        <v>100gm:—</v>
+        <v>100ml:16.54</v>
       </c>
       <c r="I16" t="str">
         <v>daily-delight-moisturising-cream</v>
@@ -1051,7 +1051,7 @@
         <v>500ml</v>
       </c>
       <c r="H17" t="str">
-        <v>500ml:—</v>
+        <v>500ml:24.3</v>
       </c>
       <c r="I17" t="str">
         <v>ice-blast-shower-gel</v>
@@ -1086,7 +1086,7 @@
         <v>100ml</v>
       </c>
       <c r="H18" t="str">
-        <v>100ml:—</v>
+        <v>100ml:28.35</v>
       </c>
       <c r="I18" t="str">
         <v>intimate-wash</v>
@@ -1156,7 +1156,7 @@
         <v>100ml, 350ml</v>
       </c>
       <c r="H20" t="str">
-        <v>100ml:—  350ml:—</v>
+        <v>100ml:8.78  350ml:21.6</v>
       </c>
       <c r="I20" t="str">
         <v>mix-fruit-body-lotion</v>
@@ -1191,7 +1191,7 @@
         <v>100ml</v>
       </c>
       <c r="H21" t="str">
-        <v>100ml:—</v>
+        <v>100ml:11.48</v>
       </c>
       <c r="I21" t="str">
         <v>mix-fruit-moisturising-cream</v>
@@ -1261,7 +1261,7 @@
         <v>500ml</v>
       </c>
       <c r="H23" t="str">
-        <v>500ml:—</v>
+        <v>500ml:24.3</v>
       </c>
       <c r="I23" t="str">
         <v>morning-buzz-shower-gel</v>
@@ -1331,7 +1331,7 @@
         <v>100ml, 400ml</v>
       </c>
       <c r="H25" t="str">
-        <v>100ml:—  400ml:—</v>
+        <v>100ml:8.44  400ml:19.24</v>
       </c>
       <c r="I25" t="str">
         <v>onion-shampoo</v>
@@ -1401,7 +1401,7 @@
         <v>100ml</v>
       </c>
       <c r="H27" t="str">
-        <v>100ml:—</v>
+        <v>100ml:20.59</v>
       </c>
       <c r="I27" t="str">
         <v>silky-touch-hair-serum</v>
@@ -1436,7 +1436,7 @@
         <v>70ml, 250ml</v>
       </c>
       <c r="H28" t="str">
-        <v>70ml:—  250ml:—</v>
+        <v>70ml:11.48  250ml:19.58</v>
       </c>
       <c r="I28" t="str">
         <v>amber-glow-body-mist</v>
@@ -1573,10 +1573,10 @@
         <v>1</v>
       </c>
       <c r="G32" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="H32" t="str">
-        <v>60ml:—</v>
+        <v>50ml:9.11</v>
       </c>
       <c r="I32" t="str">
         <v>apex-72h-roll-on</v>
@@ -1681,7 +1681,7 @@
         <v>70ml, 250ml</v>
       </c>
       <c r="H35" t="str">
-        <v>70ml:—  250ml:—</v>
+        <v>70ml:11.48  250ml:19.58</v>
       </c>
       <c r="I35" t="str">
         <v>blossom-veil-body-mist</v>
@@ -1716,7 +1716,7 @@
         <v>70ml, 250ml</v>
       </c>
       <c r="H36" t="str">
-        <v>70ml:—  250ml:—</v>
+        <v>70ml:11.48  250ml:19.58</v>
       </c>
       <c r="I36" t="str">
         <v>coastal-pulse-body-mist</v>
@@ -1818,10 +1818,10 @@
         <v>1</v>
       </c>
       <c r="G39" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="H39" t="str">
-        <v>60ml:—</v>
+        <v>50ml:9.11</v>
       </c>
       <c r="I39" t="str">
         <v>element-zero-roll-on</v>
@@ -2028,10 +2028,10 @@
         <v>1</v>
       </c>
       <c r="G45" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="H45" t="str">
-        <v>60ml:—</v>
+        <v>50ml:9.11</v>
       </c>
       <c r="I45" t="str">
         <v>lumi-glow-roll-on</v>
@@ -2066,7 +2066,7 @@
         <v>70ml, 250ml</v>
       </c>
       <c r="H46" t="str">
-        <v>70ml:—  250ml:—</v>
+        <v>70ml:11.48  250ml:19.58</v>
       </c>
       <c r="I46" t="str">
         <v>midnight-velvet-body-mist</v>
@@ -2171,7 +2171,7 @@
         <v>70ml, 250ml</v>
       </c>
       <c r="H49" t="str">
-        <v>70ml:—  250ml:—</v>
+        <v>70ml:11.48  250ml:19.58</v>
       </c>
       <c r="I49" t="str">
         <v>noir-element-body-mist</v>
@@ -2238,10 +2238,10 @@
         <v>1</v>
       </c>
       <c r="G51" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="H51" t="str">
-        <v>60ml:—</v>
+        <v>50ml:9.11</v>
       </c>
       <c r="I51" t="str">
         <v>noir-oud-roll-on</v>
@@ -2416,7 +2416,7 @@
         <v>70gm</v>
       </c>
       <c r="H56" t="str">
-        <v>70gm:—</v>
+        <v>70gm:19.58</v>
       </c>
       <c r="I56" t="str">
         <v>pure-fresh-deo-stick</v>
@@ -2448,10 +2448,10 @@
         <v>1</v>
       </c>
       <c r="G57" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="H57" t="str">
-        <v>60ml:—</v>
+        <v>50ml:9.11</v>
       </c>
       <c r="I57" t="str">
         <v>pure-renewal-roll-on</v>
@@ -2626,7 +2626,7 @@
         <v>70gm</v>
       </c>
       <c r="H62" t="str">
-        <v>70gm:—</v>
+        <v>70gm:19.58</v>
       </c>
       <c r="I62" t="str">
         <v>silk-bloom-deo-stick</v>
@@ -2661,7 +2661,7 @@
         <v>70gm</v>
       </c>
       <c r="H63" t="str">
-        <v>70gm:—</v>
+        <v>70gm:19.58</v>
       </c>
       <c r="I63" t="str">
         <v>ultra-fresh-deo-stick</v>
@@ -2696,7 +2696,7 @@
         <v>70ml, 250ml</v>
       </c>
       <c r="H64" t="str">
-        <v>70ml:—  250ml:—</v>
+        <v>70ml:11.48  250ml:19.58</v>
       </c>
       <c r="I64" t="str">
         <v>vanilla-aura-body-mist</v>
@@ -2728,10 +2728,10 @@
         <v>1</v>
       </c>
       <c r="G65" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="H65" t="str">
-        <v>60ml:—</v>
+        <v>50ml:9.11</v>
       </c>
       <c r="I65" t="str">
         <v>velvet-repair-roll-on</v>
@@ -2801,7 +2801,7 @@
         <v>60ml, 150ml</v>
       </c>
       <c r="H67" t="str">
-        <v>60ml:—  150ml:—</v>
+        <v>60ml:9.79  150ml:—</v>
       </c>
       <c r="I67" t="str">
         <v>aloevera-gel</v>
@@ -2836,7 +2836,7 @@
         <v>50ml, 150ml</v>
       </c>
       <c r="H68" t="str">
-        <v>50ml:—  150ml:—</v>
+        <v>50ml:9.79  150ml:—</v>
       </c>
       <c r="I68" t="str">
         <v>apricot-face-scrub</v>
@@ -2906,7 +2906,7 @@
         <v>50ml, 150ml</v>
       </c>
       <c r="H70" t="str">
-        <v>50ml:—  150ml:—</v>
+        <v>50ml:9.79  150ml:—</v>
       </c>
       <c r="I70" t="str">
         <v>coffee-face-scrub</v>
@@ -2941,7 +2941,7 @@
         <v>100ml, 150ml</v>
       </c>
       <c r="H71" t="str">
-        <v>100ml:—  150ml:—</v>
+        <v>100ml:17.89  150ml:—</v>
       </c>
       <c r="I71" t="str">
         <v>peel-off-mask</v>
@@ -2976,7 +2976,7 @@
         <v>100ml, 240ml</v>
       </c>
       <c r="H72" t="str">
-        <v>100ml:—  240ml:—</v>
+        <v>100ml:8.78  240ml:12.83</v>
       </c>
       <c r="I72" t="str">
         <v>rose-water-premium</v>
@@ -3081,7 +3081,7 @@
         <v>50ml, 100ml, 150ml</v>
       </c>
       <c r="H75" t="str">
-        <v>50ml:—  100ml:—  150ml:—</v>
+        <v>50ml:17.55  100ml:—  150ml:—</v>
       </c>
       <c r="I75" t="str">
         <v>sunscreen-cream</v>
@@ -3116,7 +3116,7 @@
         <v>150ml</v>
       </c>
       <c r="H76" t="str">
-        <v>150ml:—</v>
+        <v>150ml:25.65</v>
       </c>
       <c r="I76" t="str">
         <v>vit-c-foaming-face-wash</v>
@@ -3151,7 +3151,7 @@
         <v>60ml, 150ml</v>
       </c>
       <c r="H77" t="str">
-        <v>60ml:—  150ml:—</v>
+        <v>60ml:8.44  150ml:—</v>
       </c>
       <c r="I77" t="str">
         <v>vit-c-lemon-face-wash</v>
@@ -3186,7 +3186,7 @@
         <v>60ml, 150ml</v>
       </c>
       <c r="H78" t="str">
-        <v>60ml:—  150ml:—</v>
+        <v>60ml:10.13  150ml:—</v>
       </c>
       <c r="I78" t="str">
         <v>vit-c-orange-face-wash</v>
@@ -3221,7 +3221,7 @@
         <v>60ml, 150ml</v>
       </c>
       <c r="H79" t="str">
-        <v>60ml:—  150ml:—</v>
+        <v>60ml:10.13  150ml:—</v>
       </c>
       <c r="I79" t="str">
         <v>vit-c-papaya-face-wash</v>
@@ -3256,7 +3256,7 @@
         <v>50ml, 150ml</v>
       </c>
       <c r="H80" t="str">
-        <v>50ml:—  150ml:—</v>
+        <v>50ml:10.13  150ml:—</v>
       </c>
       <c r="I80" t="str">
         <v>walnut-apricot-face-scrub</v>
@@ -3291,7 +3291,7 @@
         <v>50ml, 150ml</v>
       </c>
       <c r="H81" t="str">
-        <v>50ml:—  150ml:—</v>
+        <v>50ml:9.79  150ml:—</v>
       </c>
       <c r="I81" t="str">
         <v>walnut-face-scrub</v>
@@ -3326,7 +3326,7 @@
         <v>5L</v>
       </c>
       <c r="H82" t="str">
-        <v>5L:30</v>
+        <v>5L:14.38</v>
       </c>
       <c r="I82" t="str">
         <v>3x-power-clean-citrus-burst</v>
@@ -3361,7 +3361,7 @@
         <v>3L</v>
       </c>
       <c r="H83" t="str">
-        <v>3L:22</v>
+        <v>3L:11.56</v>
       </c>
       <c r="I83" t="str">
         <v>3x-power-clean-lavender-floor-disinfectant-cleaner</v>
@@ -3396,7 +3396,7 @@
         <v>3L</v>
       </c>
       <c r="H84" t="str">
-        <v>3L:22</v>
+        <v>3L:11.56</v>
       </c>
       <c r="I84" t="str">
         <v>3x-power-clean-pine-floor-disinfectant-cleaner</v>
@@ -3431,7 +3431,7 @@
         <v>2L, 3L</v>
       </c>
       <c r="H85" t="str">
-        <v>2L:17  3L:23</v>
+        <v>2L:12.81  3L:17.19</v>
       </c>
       <c r="I85" t="str">
         <v>9x-power-clean-ultra-freshness</v>
@@ -3466,7 +3466,7 @@
         <v>3L, 5L</v>
       </c>
       <c r="H86" t="str">
-        <v>3L:24  5L:35</v>
+        <v>3L:16.88  5L:21.56</v>
       </c>
       <c r="I86" t="str">
         <v>abaya-wash</v>
@@ -3501,7 +3501,7 @@
         <v>750ml</v>
       </c>
       <c r="H87" t="str">
-        <v>750ml:13</v>
+        <v>750ml:9.06</v>
       </c>
       <c r="I87" t="str">
         <v>all-purpose-baking-soda</v>
@@ -3536,7 +3536,7 @@
         <v>1L, 3.78L</v>
       </c>
       <c r="H88" t="str">
-        <v>1L:8  3.78L:17</v>
+        <v>1L:5.31  3.78L:10.63</v>
       </c>
       <c r="I88" t="str">
         <v>bleach</v>
@@ -3571,7 +3571,7 @@
         <v>1L, 500ml</v>
       </c>
       <c r="H89" t="str">
-        <v>1L:18  500ml:12</v>
+        <v>1L:7.81  500ml:—</v>
       </c>
       <c r="I89" t="str">
         <v>cherry-blossom-handwash</v>
@@ -3606,7 +3606,7 @@
         <v>1 Kg</v>
       </c>
       <c r="H90" t="str">
-        <v>1 Kg:19</v>
+        <v>1 Kg:10.31</v>
       </c>
       <c r="I90" t="str">
         <v>citrus-burst-cleaning-gel</v>
@@ -3641,7 +3641,7 @@
         <v>5L</v>
       </c>
       <c r="H91" t="str">
-        <v>5L:28</v>
+        <v>5L:13.75</v>
       </c>
       <c r="I91" t="str">
         <v>dishwashing-liquid-aloe-and-mint-fresh</v>
@@ -3676,7 +3676,7 @@
         <v>5L</v>
       </c>
       <c r="H92" t="str">
-        <v>5L:28</v>
+        <v>5L:17.81</v>
       </c>
       <c r="I92" t="str">
         <v>dishwashing-liquid-apple-breeze</v>
@@ -3711,7 +3711,7 @@
         <v>1L, 5L</v>
       </c>
       <c r="H93" t="str">
-        <v>1L:10  5L:28</v>
+        <v>1L:4.06  5L:14.06</v>
       </c>
       <c r="I93" t="str">
         <v>dishwashing-liquid-lemon-fresh</v>
@@ -3746,7 +3746,7 @@
         <v>3L</v>
       </c>
       <c r="H94" t="str">
-        <v>3L:20</v>
+        <v>3L:13.75</v>
       </c>
       <c r="I94" t="str">
         <v>fabric-softener-relaxing-lavender</v>
@@ -3781,7 +3781,7 @@
         <v>3L</v>
       </c>
       <c r="H95" t="str">
-        <v>3L:20</v>
+        <v>3L:13.75</v>
       </c>
       <c r="I95" t="str">
         <v>fabric-softener-soft-floral-scents</v>
@@ -3816,7 +3816,7 @@
         <v>750ml</v>
       </c>
       <c r="H96" t="str">
-        <v>750ml:11</v>
+        <v>750ml:5.31</v>
       </c>
       <c r="I96" t="str">
         <v>glass-and-surface-cleaner</v>
@@ -3851,7 +3851,7 @@
         <v>1 Kg</v>
       </c>
       <c r="H97" t="str">
-        <v>1 Kg:19</v>
+        <v>1 Kg:10.31</v>
       </c>
       <c r="I97" t="str">
         <v>lavender-cleaning-gel</v>
@@ -3886,7 +3886,7 @@
         <v>5L</v>
       </c>
       <c r="H98" t="str">
-        <v>5L:26</v>
+        <v>5L:13.75</v>
       </c>
       <c r="I98" t="str">
         <v>lavender-handwash</v>
@@ -3921,7 +3921,7 @@
         <v>1L, 750ml</v>
       </c>
       <c r="H99" t="str">
-        <v>1L:19  750ml:15</v>
+        <v>1L:9.06  750ml:7.81</v>
       </c>
       <c r="I99" t="str">
         <v>lemon-fresh-multi-purpose-cream-cleaner</v>
@@ -3956,7 +3956,7 @@
         <v>5L</v>
       </c>
       <c r="H100" t="str">
-        <v>5L:26</v>
+        <v>5L:14.38</v>
       </c>
       <c r="I100" t="str">
         <v>mint-handwash</v>
@@ -3991,7 +3991,7 @@
         <v>5L</v>
       </c>
       <c r="H101" t="str">
-        <v>5L:29</v>
+        <v>5L:13.75</v>
       </c>
       <c r="I101" t="str">
         <v>oud-handwash</v>
@@ -4026,7 +4026,7 @@
         <v>5L</v>
       </c>
       <c r="H102" t="str">
-        <v>5L:26</v>
+        <v>5L:15.31</v>
       </c>
       <c r="I102" t="str">
         <v>papaya-handwash</v>
@@ -4061,7 +4061,7 @@
         <v>5L, 750ml</v>
       </c>
       <c r="H103" t="str">
-        <v>5L:32  750ml:14</v>
+        <v>5L:17.81  750ml:6.56</v>
       </c>
       <c r="I103" t="str">
         <v>pure-shield-disinfectant-cleaner</v>
@@ -4096,7 +4096,7 @@
         <v>1L, 500ml</v>
       </c>
       <c r="H104" t="str">
-        <v>1L:18  500ml:12</v>
+        <v>1L:7.81  500ml:—</v>
       </c>
       <c r="I104" t="str">
         <v>rich-musk-handwash</v>
@@ -4131,7 +4131,7 @@
         <v>1L, 500ml</v>
       </c>
       <c r="H105" t="str">
-        <v>1L:18  500ml:12</v>
+        <v>1L:7.81  500ml:—</v>
       </c>
       <c r="I105" t="str">
         <v>sweet-vanilla-handwash</v>
@@ -4166,7 +4166,7 @@
         <v>750ml</v>
       </c>
       <c r="H106" t="str">
-        <v>750ml:12</v>
+        <v>750ml:6.56</v>
       </c>
       <c r="I106" t="str">
         <v>ultra-clean-toilet-cleaner-aqua</v>
@@ -4201,7 +4201,7 @@
         <v>750ml</v>
       </c>
       <c r="H107" t="str">
-        <v>750ml:12</v>
+        <v>750ml:6.56</v>
       </c>
       <c r="I107" t="str">
         <v>ultra-clean-toilet-cleaner-pine</v>
@@ -4320,8 +4320,8 @@
       <c r="L2" t="str">
         <v/>
       </c>
-      <c r="M2" t="str">
-        <v/>
+      <c r="M2">
+        <v>23.29</v>
       </c>
       <c r="N2" t="str">
         <v/>
@@ -4379,8 +4379,8 @@
       <c r="L3" t="str">
         <v/>
       </c>
-      <c r="M3" t="str">
-        <v/>
+      <c r="M3">
+        <v>31.39</v>
       </c>
       <c r="N3" t="str">
         <v/>
@@ -4438,8 +4438,8 @@
       <c r="L4" t="str">
         <v/>
       </c>
-      <c r="M4" t="str">
-        <v/>
+      <c r="M4">
+        <v>16.88</v>
       </c>
       <c r="N4" t="str">
         <v/>
@@ -4497,8 +4497,8 @@
       <c r="L5" t="str">
         <v/>
       </c>
-      <c r="M5" t="str">
-        <v/>
+      <c r="M5">
+        <v>20.59</v>
       </c>
       <c r="N5" t="str">
         <v/>
@@ -4556,8 +4556,8 @@
       <c r="L6" t="str">
         <v/>
       </c>
-      <c r="M6" t="str">
-        <v/>
+      <c r="M6">
+        <v>11.48</v>
       </c>
       <c r="N6" t="str">
         <v/>
@@ -4615,8 +4615,8 @@
       <c r="L7" t="str">
         <v/>
       </c>
-      <c r="M7" t="str">
-        <v/>
+      <c r="M7">
+        <v>18.23</v>
       </c>
       <c r="N7" t="str">
         <v/>
@@ -4674,8 +4674,8 @@
       <c r="L8" t="str">
         <v/>
       </c>
-      <c r="M8" t="str">
-        <v/>
+      <c r="M8">
+        <v>32.4</v>
       </c>
       <c r="N8" t="str">
         <v/>
@@ -4733,8 +4733,8 @@
       <c r="L9" t="str">
         <v/>
       </c>
-      <c r="M9" t="str">
-        <v/>
+      <c r="M9">
+        <v>25.65</v>
       </c>
       <c r="N9" t="str">
         <v/>
@@ -4792,8 +4792,8 @@
       <c r="L10" t="str">
         <v/>
       </c>
-      <c r="M10" t="str">
-        <v/>
+      <c r="M10">
+        <v>31.39</v>
       </c>
       <c r="N10" t="str">
         <v/>
@@ -4851,8 +4851,8 @@
       <c r="L11" t="str">
         <v/>
       </c>
-      <c r="M11" t="str">
-        <v/>
+      <c r="M11">
+        <v>9.79</v>
       </c>
       <c r="N11" t="str">
         <v/>
@@ -4910,8 +4910,8 @@
       <c r="L12" t="str">
         <v/>
       </c>
-      <c r="M12" t="str">
-        <v/>
+      <c r="M12">
+        <v>21.6</v>
       </c>
       <c r="N12" t="str">
         <v/>
@@ -4969,8 +4969,8 @@
       <c r="L13" t="str">
         <v/>
       </c>
-      <c r="M13" t="str">
-        <v/>
+      <c r="M13">
+        <v>9.79</v>
       </c>
       <c r="N13" t="str">
         <v/>
@@ -5028,8 +5028,8 @@
       <c r="L14" t="str">
         <v/>
       </c>
-      <c r="M14" t="str">
-        <v/>
+      <c r="M14">
+        <v>24.3</v>
       </c>
       <c r="N14" t="str">
         <v/>
@@ -5087,8 +5087,8 @@
       <c r="L15" t="str">
         <v/>
       </c>
-      <c r="M15" t="str">
-        <v/>
+      <c r="M15">
+        <v>8.78</v>
       </c>
       <c r="N15" t="str">
         <v/>
@@ -5146,8 +5146,8 @@
       <c r="L16" t="str">
         <v/>
       </c>
-      <c r="M16" t="str">
-        <v/>
+      <c r="M16">
+        <v>19.24</v>
       </c>
       <c r="N16" t="str">
         <v/>
@@ -5205,8 +5205,8 @@
       <c r="L17" t="str">
         <v/>
       </c>
-      <c r="M17" t="str">
-        <v/>
+      <c r="M17">
+        <v>8.78</v>
       </c>
       <c r="N17" t="str">
         <v/>
@@ -5264,8 +5264,8 @@
       <c r="L18" t="str">
         <v/>
       </c>
-      <c r="M18" t="str">
-        <v/>
+      <c r="M18">
+        <v>22.28</v>
       </c>
       <c r="N18" t="str">
         <v/>
@@ -5323,8 +5323,8 @@
       <c r="L19" t="str">
         <v/>
       </c>
-      <c r="M19" t="str">
-        <v/>
+      <c r="M19">
+        <v>12.49</v>
       </c>
       <c r="N19" t="str">
         <v/>
@@ -5382,8 +5382,8 @@
       <c r="L20" t="str">
         <v/>
       </c>
-      <c r="M20" t="str">
-        <v/>
+      <c r="M20">
+        <v>17.89</v>
       </c>
       <c r="N20" t="str">
         <v/>
@@ -5441,8 +5441,8 @@
       <c r="L21" t="str">
         <v/>
       </c>
-      <c r="M21" t="str">
-        <v/>
+      <c r="M21">
+        <v>8.78</v>
       </c>
       <c r="N21" t="str">
         <v/>
@@ -5500,8 +5500,8 @@
       <c r="L22" t="str">
         <v/>
       </c>
-      <c r="M22" t="str">
-        <v/>
+      <c r="M22">
+        <v>18.23</v>
       </c>
       <c r="N22" t="str">
         <v/>
@@ -5559,8 +5559,8 @@
       <c r="L23" t="str">
         <v/>
       </c>
-      <c r="M23" t="str">
-        <v/>
+      <c r="M23">
+        <v>8.78</v>
       </c>
       <c r="N23" t="str">
         <v/>
@@ -5618,8 +5618,8 @@
       <c r="L24" t="str">
         <v/>
       </c>
-      <c r="M24" t="str">
-        <v/>
+      <c r="M24">
+        <v>21.6</v>
       </c>
       <c r="N24" t="str">
         <v/>
@@ -5677,8 +5677,8 @@
       <c r="L25" t="str">
         <v/>
       </c>
-      <c r="M25" t="str">
-        <v/>
+      <c r="M25">
+        <v>24.3</v>
       </c>
       <c r="N25" t="str">
         <v/>
@@ -5710,7 +5710,7 @@
         <v>JDDC100</v>
       </c>
       <c r="D26" t="str">
-        <v>Daily Delight Moisturising Cream 100gm</v>
+        <v>Daily Delight Moisturising Cream 100ml</v>
       </c>
       <c r="E26" t="str">
         <v>Daily Delight Moisturising Cream</v>
@@ -5728,7 +5728,7 @@
         <v>Body Cream</v>
       </c>
       <c r="J26" t="str">
-        <v>100gm</v>
+        <v>100ml</v>
       </c>
       <c r="K26" t="str">
         <v/>
@@ -5736,8 +5736,8 @@
       <c r="L26" t="str">
         <v/>
       </c>
-      <c r="M26" t="str">
-        <v/>
+      <c r="M26">
+        <v>16.54</v>
       </c>
       <c r="N26" t="str">
         <v/>
@@ -5795,8 +5795,8 @@
       <c r="L27" t="str">
         <v/>
       </c>
-      <c r="M27" t="str">
-        <v/>
+      <c r="M27">
+        <v>24.3</v>
       </c>
       <c r="N27" t="str">
         <v/>
@@ -5854,8 +5854,8 @@
       <c r="L28" t="str">
         <v/>
       </c>
-      <c r="M28" t="str">
-        <v/>
+      <c r="M28">
+        <v>28.35</v>
       </c>
       <c r="N28" t="str">
         <v/>
@@ -5913,9 +5913,6 @@
       <c r="L29" t="str">
         <v/>
       </c>
-      <c r="M29" t="str">
-        <v/>
-      </c>
       <c r="N29" t="str">
         <v/>
       </c>
@@ -5972,9 +5969,6 @@
       <c r="L30" t="str">
         <v/>
       </c>
-      <c r="M30" t="str">
-        <v/>
-      </c>
       <c r="N30" t="str">
         <v/>
       </c>
@@ -6031,8 +6025,8 @@
       <c r="L31" t="str">
         <v/>
       </c>
-      <c r="M31" t="str">
-        <v/>
+      <c r="M31">
+        <v>8.78</v>
       </c>
       <c r="N31" t="str">
         <v/>
@@ -6090,8 +6084,8 @@
       <c r="L32" t="str">
         <v/>
       </c>
-      <c r="M32" t="str">
-        <v/>
+      <c r="M32">
+        <v>21.6</v>
       </c>
       <c r="N32" t="str">
         <v/>
@@ -6149,8 +6143,8 @@
       <c r="L33" t="str">
         <v/>
       </c>
-      <c r="M33" t="str">
-        <v/>
+      <c r="M33">
+        <v>11.48</v>
       </c>
       <c r="N33" t="str">
         <v/>
@@ -6208,9 +6202,6 @@
       <c r="L34" t="str">
         <v/>
       </c>
-      <c r="M34" t="str">
-        <v/>
-      </c>
       <c r="N34" t="str">
         <v/>
       </c>
@@ -6267,8 +6258,8 @@
       <c r="L35" t="str">
         <v/>
       </c>
-      <c r="M35" t="str">
-        <v/>
+      <c r="M35">
+        <v>24.3</v>
       </c>
       <c r="N35" t="str">
         <v/>
@@ -6326,9 +6317,6 @@
       <c r="L36" t="str">
         <v/>
       </c>
-      <c r="M36" t="str">
-        <v/>
-      </c>
       <c r="N36" t="str">
         <v/>
       </c>
@@ -6385,8 +6373,8 @@
       <c r="L37" t="str">
         <v/>
       </c>
-      <c r="M37" t="str">
-        <v/>
+      <c r="M37">
+        <v>8.44</v>
       </c>
       <c r="N37" t="str">
         <v/>
@@ -6444,8 +6432,8 @@
       <c r="L38" t="str">
         <v/>
       </c>
-      <c r="M38" t="str">
-        <v/>
+      <c r="M38">
+        <v>19.24</v>
       </c>
       <c r="N38" t="str">
         <v/>
@@ -6503,9 +6491,6 @@
       <c r="L39" t="str">
         <v/>
       </c>
-      <c r="M39" t="str">
-        <v/>
-      </c>
       <c r="N39" t="str">
         <v/>
       </c>
@@ -6562,8 +6547,8 @@
       <c r="L40" t="str">
         <v/>
       </c>
-      <c r="M40" t="str">
-        <v/>
+      <c r="M40">
+        <v>20.59</v>
       </c>
       <c r="N40" t="str">
         <v/>
@@ -6621,8 +6606,8 @@
       <c r="L41" t="str">
         <v/>
       </c>
-      <c r="M41" t="str">
-        <v/>
+      <c r="M41">
+        <v>11.48</v>
       </c>
       <c r="N41" t="str">
         <v/>
@@ -6680,8 +6665,8 @@
       <c r="L42" t="str">
         <v/>
       </c>
-      <c r="M42" t="str">
-        <v/>
+      <c r="M42">
+        <v>19.58</v>
       </c>
       <c r="N42" t="str">
         <v/>
@@ -6739,9 +6724,6 @@
       <c r="L43" t="str">
         <v/>
       </c>
-      <c r="M43" t="str">
-        <v/>
-      </c>
       <c r="N43" t="str">
         <v/>
       </c>
@@ -6798,9 +6780,6 @@
       <c r="L44" t="str">
         <v/>
       </c>
-      <c r="M44" t="str">
-        <v/>
-      </c>
       <c r="N44" t="str">
         <v/>
       </c>
@@ -6857,9 +6836,6 @@
       <c r="L45" t="str">
         <v/>
       </c>
-      <c r="M45" t="str">
-        <v/>
-      </c>
       <c r="N45" t="str">
         <v/>
       </c>
@@ -6890,7 +6866,7 @@
         <v>#00681</v>
       </c>
       <c r="D46" t="str">
-        <v>Apex 72H Roll On 60ml</v>
+        <v>Apex 72H Roll On 50ml</v>
       </c>
       <c r="E46" t="str">
         <v>Apex 72H Roll On</v>
@@ -6908,7 +6884,7 @@
         <v>Roll On</v>
       </c>
       <c r="J46" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -6916,8 +6892,8 @@
       <c r="L46" t="str">
         <v/>
       </c>
-      <c r="M46" t="str">
-        <v/>
+      <c r="M46">
+        <v>9.11</v>
       </c>
       <c r="N46" t="str">
         <v/>
@@ -6975,9 +6951,6 @@
       <c r="L47" t="str">
         <v/>
       </c>
-      <c r="M47" t="str">
-        <v/>
-      </c>
       <c r="N47" t="str">
         <v/>
       </c>
@@ -7034,9 +7007,6 @@
       <c r="L48" t="str">
         <v/>
       </c>
-      <c r="M48" t="str">
-        <v/>
-      </c>
       <c r="N48" t="str">
         <v/>
       </c>
@@ -7093,8 +7063,8 @@
       <c r="L49" t="str">
         <v/>
       </c>
-      <c r="M49" t="str">
-        <v/>
+      <c r="M49">
+        <v>11.48</v>
       </c>
       <c r="N49" t="str">
         <v/>
@@ -7152,8 +7122,8 @@
       <c r="L50" t="str">
         <v/>
       </c>
-      <c r="M50" t="str">
-        <v/>
+      <c r="M50">
+        <v>19.58</v>
       </c>
       <c r="N50" t="str">
         <v/>
@@ -7211,8 +7181,8 @@
       <c r="L51" t="str">
         <v/>
       </c>
-      <c r="M51" t="str">
-        <v/>
+      <c r="M51">
+        <v>11.48</v>
       </c>
       <c r="N51" t="str">
         <v/>
@@ -7270,8 +7240,8 @@
       <c r="L52" t="str">
         <v/>
       </c>
-      <c r="M52" t="str">
-        <v/>
+      <c r="M52">
+        <v>19.58</v>
       </c>
       <c r="N52" t="str">
         <v/>
@@ -7329,9 +7299,6 @@
       <c r="L53" t="str">
         <v/>
       </c>
-      <c r="M53" t="str">
-        <v/>
-      </c>
       <c r="N53" t="str">
         <v/>
       </c>
@@ -7388,9 +7355,6 @@
       <c r="L54" t="str">
         <v/>
       </c>
-      <c r="M54" t="str">
-        <v/>
-      </c>
       <c r="N54" t="str">
         <v/>
       </c>
@@ -7421,7 +7385,7 @@
         <v>#00683</v>
       </c>
       <c r="D55" t="str">
-        <v>Element Zero Roll On 60ml</v>
+        <v>Element Zero Roll On 50ml</v>
       </c>
       <c r="E55" t="str">
         <v>Element Zero Roll On</v>
@@ -7439,7 +7403,7 @@
         <v>Roll On</v>
       </c>
       <c r="J55" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="K55" t="str">
         <v/>
@@ -7447,8 +7411,8 @@
       <c r="L55" t="str">
         <v/>
       </c>
-      <c r="M55" t="str">
-        <v/>
+      <c r="M55">
+        <v>9.11</v>
       </c>
       <c r="N55" t="str">
         <v/>
@@ -7506,9 +7470,6 @@
       <c r="L56" t="str">
         <v/>
       </c>
-      <c r="M56" t="str">
-        <v/>
-      </c>
       <c r="N56" t="str">
         <v/>
       </c>
@@ -7565,9 +7526,6 @@
       <c r="L57" t="str">
         <v/>
       </c>
-      <c r="M57" t="str">
-        <v/>
-      </c>
       <c r="N57" t="str">
         <v/>
       </c>
@@ -7624,9 +7582,6 @@
       <c r="L58" t="str">
         <v/>
       </c>
-      <c r="M58" t="str">
-        <v/>
-      </c>
       <c r="N58" t="str">
         <v/>
       </c>
@@ -7683,9 +7638,6 @@
       <c r="L59" t="str">
         <v/>
       </c>
-      <c r="M59" t="str">
-        <v/>
-      </c>
       <c r="N59" t="str">
         <v/>
       </c>
@@ -7742,9 +7694,6 @@
       <c r="L60" t="str">
         <v/>
       </c>
-      <c r="M60" t="str">
-        <v/>
-      </c>
       <c r="N60" t="str">
         <v/>
       </c>
@@ -7775,7 +7724,7 @@
         <v>#00678</v>
       </c>
       <c r="D61" t="str">
-        <v>Lumi Glow Roll On 60ml</v>
+        <v>Lumi Glow Roll On 50ml</v>
       </c>
       <c r="E61" t="str">
         <v>Lumi Glow Roll On</v>
@@ -7793,7 +7742,7 @@
         <v>Roll On</v>
       </c>
       <c r="J61" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="K61" t="str">
         <v/>
@@ -7801,8 +7750,8 @@
       <c r="L61" t="str">
         <v/>
       </c>
-      <c r="M61" t="str">
-        <v/>
+      <c r="M61">
+        <v>9.11</v>
       </c>
       <c r="N61" t="str">
         <v/>
@@ -7860,8 +7809,8 @@
       <c r="L62" t="str">
         <v/>
       </c>
-      <c r="M62" t="str">
-        <v/>
+      <c r="M62">
+        <v>11.48</v>
       </c>
       <c r="N62" t="str">
         <v/>
@@ -7919,8 +7868,8 @@
       <c r="L63" t="str">
         <v/>
       </c>
-      <c r="M63" t="str">
-        <v/>
+      <c r="M63">
+        <v>19.58</v>
       </c>
       <c r="N63" t="str">
         <v/>
@@ -7978,9 +7927,6 @@
       <c r="L64" t="str">
         <v/>
       </c>
-      <c r="M64" t="str">
-        <v/>
-      </c>
       <c r="N64" t="str">
         <v/>
       </c>
@@ -8037,9 +7983,6 @@
       <c r="L65" t="str">
         <v/>
       </c>
-      <c r="M65" t="str">
-        <v/>
-      </c>
       <c r="N65" t="str">
         <v/>
       </c>
@@ -8096,8 +8039,8 @@
       <c r="L66" t="str">
         <v/>
       </c>
-      <c r="M66" t="str">
-        <v/>
+      <c r="M66">
+        <v>11.48</v>
       </c>
       <c r="N66" t="str">
         <v/>
@@ -8155,8 +8098,8 @@
       <c r="L67" t="str">
         <v/>
       </c>
-      <c r="M67" t="str">
-        <v/>
+      <c r="M67">
+        <v>19.58</v>
       </c>
       <c r="N67" t="str">
         <v/>
@@ -8214,9 +8157,6 @@
       <c r="L68" t="str">
         <v/>
       </c>
-      <c r="M68" t="str">
-        <v/>
-      </c>
       <c r="N68" t="str">
         <v/>
       </c>
@@ -8247,7 +8187,7 @@
         <v>#00682</v>
       </c>
       <c r="D69" t="str">
-        <v>Noir Oud Roll On 60ml</v>
+        <v>Noir Oud Roll On 50ml</v>
       </c>
       <c r="E69" t="str">
         <v>Noir Oud Roll On</v>
@@ -8265,7 +8205,7 @@
         <v>Roll On</v>
       </c>
       <c r="J69" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="K69" t="str">
         <v/>
@@ -8273,8 +8213,8 @@
       <c r="L69" t="str">
         <v/>
       </c>
-      <c r="M69" t="str">
-        <v/>
+      <c r="M69">
+        <v>9.11</v>
       </c>
       <c r="N69" t="str">
         <v/>
@@ -8332,9 +8272,6 @@
       <c r="L70" t="str">
         <v/>
       </c>
-      <c r="M70" t="str">
-        <v/>
-      </c>
       <c r="N70" t="str">
         <v/>
       </c>
@@ -8391,9 +8328,6 @@
       <c r="L71" t="str">
         <v/>
       </c>
-      <c r="M71" t="str">
-        <v/>
-      </c>
       <c r="N71" t="str">
         <v/>
       </c>
@@ -8450,9 +8384,6 @@
       <c r="L72" t="str">
         <v/>
       </c>
-      <c r="M72" t="str">
-        <v/>
-      </c>
       <c r="N72" t="str">
         <v/>
       </c>
@@ -8509,9 +8440,6 @@
       <c r="L73" t="str">
         <v/>
       </c>
-      <c r="M73" t="str">
-        <v/>
-      </c>
       <c r="N73" t="str">
         <v/>
       </c>
@@ -8568,8 +8496,8 @@
       <c r="L74" t="str">
         <v/>
       </c>
-      <c r="M74" t="str">
-        <v/>
+      <c r="M74">
+        <v>19.58</v>
       </c>
       <c r="N74" t="str">
         <v/>
@@ -8601,7 +8529,7 @@
         <v>#00680</v>
       </c>
       <c r="D75" t="str">
-        <v>Pure Renewal Roll On 60ml</v>
+        <v>Pure Renewal Roll On 50ml</v>
       </c>
       <c r="E75" t="str">
         <v>Pure Renewal Roll On</v>
@@ -8619,7 +8547,7 @@
         <v>Roll On</v>
       </c>
       <c r="J75" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="K75" t="str">
         <v/>
@@ -8627,8 +8555,8 @@
       <c r="L75" t="str">
         <v/>
       </c>
-      <c r="M75" t="str">
-        <v/>
+      <c r="M75">
+        <v>9.11</v>
       </c>
       <c r="N75" t="str">
         <v/>
@@ -8686,9 +8614,6 @@
       <c r="L76" t="str">
         <v/>
       </c>
-      <c r="M76" t="str">
-        <v/>
-      </c>
       <c r="N76" t="str">
         <v/>
       </c>
@@ -8745,9 +8670,6 @@
       <c r="L77" t="str">
         <v/>
       </c>
-      <c r="M77" t="str">
-        <v/>
-      </c>
       <c r="N77" t="str">
         <v/>
       </c>
@@ -8804,9 +8726,6 @@
       <c r="L78" t="str">
         <v/>
       </c>
-      <c r="M78" t="str">
-        <v/>
-      </c>
       <c r="N78" t="str">
         <v/>
       </c>
@@ -8863,9 +8782,6 @@
       <c r="L79" t="str">
         <v/>
       </c>
-      <c r="M79" t="str">
-        <v/>
-      </c>
       <c r="N79" t="str">
         <v/>
       </c>
@@ -8922,8 +8838,8 @@
       <c r="L80" t="str">
         <v/>
       </c>
-      <c r="M80" t="str">
-        <v/>
+      <c r="M80">
+        <v>19.58</v>
       </c>
       <c r="N80" t="str">
         <v/>
@@ -8981,8 +8897,8 @@
       <c r="L81" t="str">
         <v/>
       </c>
-      <c r="M81" t="str">
-        <v/>
+      <c r="M81">
+        <v>19.58</v>
       </c>
       <c r="N81" t="str">
         <v/>
@@ -9040,8 +8956,8 @@
       <c r="L82" t="str">
         <v/>
       </c>
-      <c r="M82" t="str">
-        <v/>
+      <c r="M82">
+        <v>11.48</v>
       </c>
       <c r="N82" t="str">
         <v/>
@@ -9099,8 +9015,8 @@
       <c r="L83" t="str">
         <v/>
       </c>
-      <c r="M83" t="str">
-        <v/>
+      <c r="M83">
+        <v>19.58</v>
       </c>
       <c r="N83" t="str">
         <v/>
@@ -9132,7 +9048,7 @@
         <v>#00679</v>
       </c>
       <c r="D84" t="str">
-        <v>Velvet Repair Roll On 60ml</v>
+        <v>Velvet Repair Roll On 50ml</v>
       </c>
       <c r="E84" t="str">
         <v>Velvet Repair Roll On</v>
@@ -9150,7 +9066,7 @@
         <v>Roll On</v>
       </c>
       <c r="J84" t="str">
-        <v>60ml</v>
+        <v>50ml</v>
       </c>
       <c r="K84" t="str">
         <v/>
@@ -9158,8 +9074,8 @@
       <c r="L84" t="str">
         <v/>
       </c>
-      <c r="M84" t="str">
-        <v/>
+      <c r="M84">
+        <v>9.11</v>
       </c>
       <c r="N84" t="str">
         <v/>
@@ -9217,9 +9133,6 @@
       <c r="L85" t="str">
         <v/>
       </c>
-      <c r="M85" t="str">
-        <v/>
-      </c>
       <c r="N85" t="str">
         <v/>
       </c>
@@ -9276,8 +9189,8 @@
       <c r="L86" t="str">
         <v/>
       </c>
-      <c r="M86" t="str">
-        <v/>
+      <c r="M86">
+        <v>9.79</v>
       </c>
       <c r="N86" t="str">
         <v/>
@@ -9335,9 +9248,6 @@
       <c r="L87" t="str">
         <v/>
       </c>
-      <c r="M87" t="str">
-        <v/>
-      </c>
       <c r="N87" t="str">
         <v/>
       </c>
@@ -9394,8 +9304,8 @@
       <c r="L88" t="str">
         <v/>
       </c>
-      <c r="M88" t="str">
-        <v/>
+      <c r="M88">
+        <v>9.79</v>
       </c>
       <c r="N88" t="str">
         <v/>
@@ -9453,9 +9363,6 @@
       <c r="L89" t="str">
         <v/>
       </c>
-      <c r="M89" t="str">
-        <v/>
-      </c>
       <c r="N89" t="str">
         <v/>
       </c>
@@ -9512,9 +9419,6 @@
       <c r="L90" t="str">
         <v/>
       </c>
-      <c r="M90" t="str">
-        <v/>
-      </c>
       <c r="N90" t="str">
         <v/>
       </c>
@@ -9571,8 +9475,8 @@
       <c r="L91" t="str">
         <v/>
       </c>
-      <c r="M91" t="str">
-        <v/>
+      <c r="M91">
+        <v>9.79</v>
       </c>
       <c r="N91" t="str">
         <v/>
@@ -9630,9 +9534,6 @@
       <c r="L92" t="str">
         <v/>
       </c>
-      <c r="M92" t="str">
-        <v/>
-      </c>
       <c r="N92" t="str">
         <v/>
       </c>
@@ -9689,8 +9590,8 @@
       <c r="L93" t="str">
         <v/>
       </c>
-      <c r="M93" t="str">
-        <v/>
+      <c r="M93">
+        <v>17.89</v>
       </c>
       <c r="N93" t="str">
         <v/>
@@ -9748,9 +9649,6 @@
       <c r="L94" t="str">
         <v/>
       </c>
-      <c r="M94" t="str">
-        <v/>
-      </c>
       <c r="N94" t="str">
         <v/>
       </c>
@@ -9807,8 +9705,8 @@
       <c r="L95" t="str">
         <v/>
       </c>
-      <c r="M95" t="str">
-        <v/>
+      <c r="M95">
+        <v>8.78</v>
       </c>
       <c r="N95" t="str">
         <v/>
@@ -9866,8 +9764,8 @@
       <c r="L96" t="str">
         <v/>
       </c>
-      <c r="M96" t="str">
-        <v/>
+      <c r="M96">
+        <v>12.83</v>
       </c>
       <c r="N96" t="str">
         <v/>
@@ -9925,9 +9823,6 @@
       <c r="L97" t="str">
         <v/>
       </c>
-      <c r="M97" t="str">
-        <v/>
-      </c>
       <c r="N97" t="str">
         <v/>
       </c>
@@ -9984,9 +9879,6 @@
       <c r="L98" t="str">
         <v/>
       </c>
-      <c r="M98" t="str">
-        <v/>
-      </c>
       <c r="N98" t="str">
         <v/>
       </c>
@@ -10043,8 +9935,8 @@
       <c r="L99" t="str">
         <v/>
       </c>
-      <c r="M99" t="str">
-        <v/>
+      <c r="M99">
+        <v>17.55</v>
       </c>
       <c r="N99" t="str">
         <v/>
@@ -10102,9 +9994,6 @@
       <c r="L100" t="str">
         <v/>
       </c>
-      <c r="M100" t="str">
-        <v/>
-      </c>
       <c r="N100" t="str">
         <v/>
       </c>
@@ -10161,9 +10050,6 @@
       <c r="L101" t="str">
         <v/>
       </c>
-      <c r="M101" t="str">
-        <v/>
-      </c>
       <c r="N101" t="str">
         <v/>
       </c>
@@ -10220,8 +10106,8 @@
       <c r="L102" t="str">
         <v/>
       </c>
-      <c r="M102" t="str">
-        <v/>
+      <c r="M102">
+        <v>25.65</v>
       </c>
       <c r="N102" t="str">
         <v/>
@@ -10279,8 +10165,8 @@
       <c r="L103" t="str">
         <v/>
       </c>
-      <c r="M103" t="str">
-        <v/>
+      <c r="M103">
+        <v>8.44</v>
       </c>
       <c r="N103" t="str">
         <v/>
@@ -10338,9 +10224,6 @@
       <c r="L104" t="str">
         <v/>
       </c>
-      <c r="M104" t="str">
-        <v/>
-      </c>
       <c r="N104" t="str">
         <v/>
       </c>
@@ -10397,8 +10280,8 @@
       <c r="L105" t="str">
         <v/>
       </c>
-      <c r="M105" t="str">
-        <v/>
+      <c r="M105">
+        <v>10.13</v>
       </c>
       <c r="N105" t="str">
         <v/>
@@ -10456,9 +10339,6 @@
       <c r="L106" t="str">
         <v/>
       </c>
-      <c r="M106" t="str">
-        <v/>
-      </c>
       <c r="N106" t="str">
         <v/>
       </c>
@@ -10515,8 +10395,8 @@
       <c r="L107" t="str">
         <v/>
       </c>
-      <c r="M107" t="str">
-        <v/>
+      <c r="M107">
+        <v>10.13</v>
       </c>
       <c r="N107" t="str">
         <v/>
@@ -10574,9 +10454,6 @@
       <c r="L108" t="str">
         <v/>
       </c>
-      <c r="M108" t="str">
-        <v/>
-      </c>
       <c r="N108" t="str">
         <v/>
       </c>
@@ -10633,8 +10510,8 @@
       <c r="L109" t="str">
         <v/>
       </c>
-      <c r="M109" t="str">
-        <v/>
+      <c r="M109">
+        <v>10.13</v>
       </c>
       <c r="N109" t="str">
         <v/>
@@ -10692,9 +10569,6 @@
       <c r="L110" t="str">
         <v/>
       </c>
-      <c r="M110" t="str">
-        <v/>
-      </c>
       <c r="N110" t="str">
         <v/>
       </c>
@@ -10751,8 +10625,8 @@
       <c r="L111" t="str">
         <v/>
       </c>
-      <c r="M111" t="str">
-        <v/>
+      <c r="M111">
+        <v>9.79</v>
       </c>
       <c r="N111" t="str">
         <v/>
@@ -10810,9 +10684,6 @@
       <c r="L112" t="str">
         <v/>
       </c>
-      <c r="M112" t="str">
-        <v/>
-      </c>
       <c r="N112" t="str">
         <v/>
       </c>
@@ -10869,8 +10740,8 @@
       <c r="L113" t="str">
         <v>Citrus Burst</v>
       </c>
-      <c r="M113" t="str">
-        <v>30</v>
+      <c r="M113">
+        <v>14.38</v>
       </c>
       <c r="N113" t="str">
         <v>Triple-action citrus-powered floor disinfectant cleaner that delivers deep cleaning, disinfecting, and a long-lasting fresh scent in one pass.</v>
@@ -10928,8 +10799,8 @@
       <c r="L114" t="str">
         <v>Lavender</v>
       </c>
-      <c r="M114" t="str">
-        <v>22</v>
+      <c r="M114">
+        <v>11.56</v>
       </c>
       <c r="N114" t="str">
         <v>Triple-action floor disinfectant cleaner with relaxing lavender fragrance for deep cleaning floors.</v>
@@ -10987,8 +10858,8 @@
       <c r="L115" t="str">
         <v>Pine</v>
       </c>
-      <c r="M115" t="str">
-        <v>22</v>
+      <c r="M115">
+        <v>11.56</v>
       </c>
       <c r="N115" t="str">
         <v>Triple-action floor disinfectant cleaner with refreshing pine fragrance for deep cleaning floors.</v>
@@ -11046,8 +10917,8 @@
       <c r="L116" t="str">
         <v>Ultra Freshness</v>
       </c>
-      <c r="M116" t="str">
-        <v>17</v>
+      <c r="M116">
+        <v>12.81</v>
       </c>
       <c r="N116" t="str">
         <v>9X power laundry liquid detergent delivering ultra freshness and deep stain removal, compact 2L size.</v>
@@ -11105,8 +10976,8 @@
       <c r="L117" t="str">
         <v>Ultra Freshness</v>
       </c>
-      <c r="M117" t="str">
-        <v>23</v>
+      <c r="M117">
+        <v>17.19</v>
       </c>
       <c r="N117" t="str">
         <v>9X power laundry liquid detergent delivering ultra freshness and deep stain removal.</v>
@@ -11164,8 +11035,8 @@
       <c r="L118" t="str">
         <v>Color &amp; Fiber Revival</v>
       </c>
-      <c r="M118" t="str">
-        <v>24</v>
+      <c r="M118">
+        <v>16.88</v>
       </c>
       <c r="N118" t="str">
         <v>Specially formulated abaya shampoo for color &amp; fiber revival with long-lasting fresh scent.</v>
@@ -11223,8 +11094,8 @@
       <c r="L119" t="str">
         <v>Color &amp; Fiber Revival</v>
       </c>
-      <c r="M119" t="str">
-        <v>35</v>
+      <c r="M119">
+        <v>21.56</v>
       </c>
       <c r="N119" t="str">
         <v>Specially formulated abaya shampoo for color &amp; fiber revival with long-lasting fresh scent, bulk 5L size.</v>
@@ -11282,8 +11153,8 @@
       <c r="L120" t="str">
         <v>Baking Soda Formula</v>
       </c>
-      <c r="M120" t="str">
-        <v>13</v>
+      <c r="M120">
+        <v>9.06</v>
       </c>
       <c r="N120" t="str">
         <v>Deep-cleaning multi-purpose cleaner powered by natural baking soda, tackles stubborn grease with a crystal-clear shine.</v>
@@ -11341,8 +11212,8 @@
       <c r="L121" t="str">
         <v>Original</v>
       </c>
-      <c r="M121" t="str">
-        <v>8</v>
+      <c r="M121">
+        <v>5.31</v>
       </c>
       <c r="N121" t="str">
         <v>High-strength multi-surface bleach for disinfecting and whitening household surfaces.</v>
@@ -11400,8 +11271,8 @@
       <c r="L122" t="str">
         <v>Original</v>
       </c>
-      <c r="M122" t="str">
-        <v>17</v>
+      <c r="M122">
+        <v>10.63</v>
       </c>
       <c r="N122" t="str">
         <v>High-strength multi-surface bleach for disinfecting and whitening, bulk 3.78L size.</v>
@@ -11459,8 +11330,8 @@
       <c r="L123" t="str">
         <v>Cherry Blossom</v>
       </c>
-      <c r="M123" t="str">
-        <v>18</v>
+      <c r="M123">
+        <v>7.81</v>
       </c>
       <c r="N123" t="str">
         <v>Premium hand wash infused with delicate cherry blossom fragrance for gentle cleansing &amp; moisturizing.</v>
@@ -11518,9 +11389,6 @@
       <c r="L124" t="str">
         <v>Cherry Blossom</v>
       </c>
-      <c r="M124" t="str">
-        <v>12</v>
-      </c>
       <c r="N124" t="str">
         <v>Premium hand wash infused with delicate cherry blossom fragrance — mid-size pump bottle, ideal for guest bathrooms.</v>
       </c>
@@ -11577,8 +11445,8 @@
       <c r="L125" t="str">
         <v>Citrus Burst</v>
       </c>
-      <c r="M125" t="str">
-        <v>19</v>
+      <c r="M125">
+        <v>10.31</v>
       </c>
       <c r="N125" t="str">
         <v>Powerful citrus cleaning gel that lifts grime while leaving a fresh citrus scent.</v>
@@ -11636,8 +11504,8 @@
       <c r="L126" t="str">
         <v>Aloe &amp; Mint Fresh</v>
       </c>
-      <c r="M126" t="str">
-        <v>28</v>
+      <c r="M126">
+        <v>13.75</v>
       </c>
       <c r="N126" t="str">
         <v>Advanced grease-cutting dishwashing liquid with aloe &amp; mint, cuts through grease &amp; leaves dishes sparkling clean.</v>
@@ -11695,8 +11563,8 @@
       <c r="L127" t="str">
         <v>Apple Breeze</v>
       </c>
-      <c r="M127" t="str">
-        <v>28</v>
+      <c r="M127">
+        <v>17.81</v>
       </c>
       <c r="N127" t="str">
         <v>Refreshing grease-cutting dishwashing liquid with apple breeze fragrance, leaves dishes sparkling clean.</v>
@@ -11754,8 +11622,8 @@
       <c r="L128" t="str">
         <v>Lemon Fresh</v>
       </c>
-      <c r="M128" t="str">
-        <v>10</v>
+      <c r="M128">
+        <v>4.06</v>
       </c>
       <c r="N128" t="str">
         <v>Ultra-concentrated lemon fresh dishwashing liquid that cuts grease fast and is gentle on hands.</v>
@@ -11813,8 +11681,8 @@
       <c r="L129" t="str">
         <v>Lemon Fresh</v>
       </c>
-      <c r="M129" t="str">
-        <v>28</v>
+      <c r="M129">
+        <v>14.06</v>
       </c>
       <c r="N129" t="str">
         <v>Powerful grease-cutting dishwashing liquid with lemon fresh fragrance, leaves dishes sparkling clean.</v>
@@ -11872,8 +11740,8 @@
       <c r="L130" t="str">
         <v>Relaxing Lavender</v>
       </c>
-      <c r="M130" t="str">
-        <v>20</v>
+      <c r="M130">
+        <v>13.75</v>
       </c>
       <c r="N130" t="str">
         <v>Fabric softener with relaxing lavender fragrance, suitable for machine &amp; hand wash with long-lasting freshness.</v>
@@ -11931,8 +11799,8 @@
       <c r="L131" t="str">
         <v>Soft Floral Scents</v>
       </c>
-      <c r="M131" t="str">
-        <v>20</v>
+      <c r="M131">
+        <v>13.75</v>
       </c>
       <c r="N131" t="str">
         <v>Fabric softener with soft floral fragrance, suitable for machine &amp; hand wash with long-lasting freshness.</v>
@@ -11990,8 +11858,8 @@
       <c r="L132" t="str">
         <v>Original</v>
       </c>
-      <c r="M132" t="str">
-        <v>11</v>
+      <c r="M132">
+        <v>5.31</v>
       </c>
       <c r="N132" t="str">
         <v>Streak-free glass and surface cleaner for a crystal-clear shine on mirrors, windows, and all glass.</v>
@@ -12049,8 +11917,8 @@
       <c r="L133" t="str">
         <v>Lavender</v>
       </c>
-      <c r="M133" t="str">
-        <v>19</v>
+      <c r="M133">
+        <v>10.31</v>
       </c>
       <c r="N133" t="str">
         <v>Thick cleaning gel infused with calming lavender for everyday surface cleaning.</v>
@@ -12108,8 +11976,8 @@
       <c r="L134" t="str">
         <v>Lavender</v>
       </c>
-      <c r="M134" t="str">
-        <v>26</v>
+      <c r="M134">
+        <v>13.75</v>
       </c>
       <c r="N134" t="str">
         <v>Advanced moisturising hand wash with calming lavender fragrance, kills 99.9% of germs &amp; bacteria. Bulk refill size.</v>
@@ -12167,8 +12035,8 @@
       <c r="L135" t="str">
         <v>Lemon</v>
       </c>
-      <c r="M135" t="str">
-        <v>19</v>
+      <c r="M135">
+        <v>9.06</v>
       </c>
       <c r="N135" t="str">
         <v>Lemon-scented cream cleaner that removes 100% of the toughest dirt with damage-free cleaning particles.</v>
@@ -12226,8 +12094,8 @@
       <c r="L136" t="str">
         <v>Lemon</v>
       </c>
-      <c r="M136" t="str">
-        <v>15</v>
+      <c r="M136">
+        <v>7.81</v>
       </c>
       <c r="N136" t="str">
         <v>Lemon-scented cream cleaner that removes 100% of the toughest dirt with damage-free cleaning particles.</v>
@@ -12285,8 +12153,8 @@
       <c r="L137" t="str">
         <v>Mint Fresh</v>
       </c>
-      <c r="M137" t="str">
-        <v>26</v>
+      <c r="M137">
+        <v>14.38</v>
       </c>
       <c r="N137" t="str">
         <v>Advanced moisturising hand wash with refreshing mint fragrance, kills 99.9% of germs &amp; bacteria. Bulk refill size.</v>
@@ -12344,8 +12212,8 @@
       <c r="L138" t="str">
         <v>Oud Royale</v>
       </c>
-      <c r="M138" t="str">
-        <v>29</v>
+      <c r="M138">
+        <v>13.75</v>
       </c>
       <c r="N138" t="str">
         <v>Advanced moisturising hand wash infused with luxurious Oud Royale fragrance, kills 99.9% of germs &amp; bacteria. Bulk refill size.</v>
@@ -12403,8 +12271,8 @@
       <c r="L139" t="str">
         <v>Papaya</v>
       </c>
-      <c r="M139" t="str">
-        <v>26</v>
+      <c r="M139">
+        <v>15.31</v>
       </c>
       <c r="N139" t="str">
         <v>Advanced moisturising hand wash with tropical papaya fragrance, kills 99.9% of germs &amp; bacteria. Bulk refill size.</v>
@@ -12462,8 +12330,8 @@
       <c r="L140" t="str">
         <v>Pure-Shield</v>
       </c>
-      <c r="M140" t="str">
-        <v>32</v>
+      <c r="M140">
+        <v>17.81</v>
       </c>
       <c r="N140" t="str">
         <v>Advanced antiseptic disinfectant cleaner that kills 99.9% of germs &amp; bacteria, bulk 5L size for homes &amp; businesses.</v>
@@ -12521,8 +12389,8 @@
       <c r="L141" t="str">
         <v>Pure-Shield</v>
       </c>
-      <c r="M141" t="str">
-        <v>14</v>
+      <c r="M141">
+        <v>6.56</v>
       </c>
       <c r="N141" t="str">
         <v>Advanced antiseptic disinfectant cleaner that kills 99.9% of germs &amp; bacteria with multi-surface protection for floors, counters, and appliances.</v>
@@ -12580,8 +12448,8 @@
       <c r="L142" t="str">
         <v>Rich Musk</v>
       </c>
-      <c r="M142" t="str">
-        <v>18</v>
+      <c r="M142">
+        <v>7.81</v>
       </c>
       <c r="N142" t="str">
         <v>Premium hand wash infused with rich musk fragrance for gentle cleansing &amp; long-lasting luxurious freshness.</v>
@@ -12639,9 +12507,6 @@
       <c r="L143" t="str">
         <v>Rich Musk</v>
       </c>
-      <c r="M143" t="str">
-        <v>12</v>
-      </c>
       <c r="N143" t="str">
         <v>Premium hand wash infused with rich musk fragrance — mid-size pump bottle, ideal for guest bathrooms.</v>
       </c>
@@ -12698,8 +12563,8 @@
       <c r="L144" t="str">
         <v>Sweet Vanilla</v>
       </c>
-      <c r="M144" t="str">
-        <v>18</v>
+      <c r="M144">
+        <v>7.81</v>
       </c>
       <c r="N144" t="str">
         <v>Premium hand wash with sweet vanilla fragrance for gentle cleansing &amp; moisturizing, made with natural ingredients.</v>
@@ -12757,9 +12622,6 @@
       <c r="L145" t="str">
         <v>Sweet Vanilla</v>
       </c>
-      <c r="M145" t="str">
-        <v>12</v>
-      </c>
       <c r="N145" t="str">
         <v>Premium hand wash with sweet vanilla fragrance for gentle cleansing &amp; moisturizing — mid-size pump bottle, ideal for guest bathrooms.</v>
       </c>
@@ -12816,8 +12678,8 @@
       <c r="L146" t="str">
         <v>Aqua Fresh</v>
       </c>
-      <c r="M146" t="str">
-        <v>12</v>
+      <c r="M146">
+        <v>6.56</v>
       </c>
       <c r="N146" t="str">
         <v>Powerful toilet cleaner with fresh aqua scent that kills 99.9% of germs and removes limescale &amp; stains.</v>
@@ -12875,8 +12737,8 @@
       <c r="L147" t="str">
         <v>Pine</v>
       </c>
-      <c r="M147" t="str">
-        <v>12</v>
+      <c r="M147">
+        <v>6.56</v>
       </c>
       <c r="N147" t="str">
         <v>Powerful toilet cleaner with fresh pine scent that kills 99.9% of germs and removes limescale.</v>

</xml_diff>